<commit_message>
Adatpt case study to 48 h
</commit_message>
<xml_diff>
--- a/data/mini-example-resilience/Heat_Demand.xlsx
+++ b/data/mini-example-resilience/Heat_Demand.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Simon Malacek\Code\LEGO-Pyomo\data\mini-example-resilience\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5487DE0A-8B12-40CB-ACFB-E452CE19DBC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF6D7F60-6F48-4EE4-9FE8-A97736E10C1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -100,7 +100,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="84">
   <si>
     <t>Heat - Demand</t>
   </si>
@@ -280,6 +280,78 @@
   </si>
   <si>
     <t>building</t>
+  </si>
+  <si>
+    <t>k0025</t>
+  </si>
+  <si>
+    <t>k0026</t>
+  </si>
+  <si>
+    <t>k0027</t>
+  </si>
+  <si>
+    <t>k0028</t>
+  </si>
+  <si>
+    <t>k0029</t>
+  </si>
+  <si>
+    <t>k0030</t>
+  </si>
+  <si>
+    <t>k0031</t>
+  </si>
+  <si>
+    <t>k0032</t>
+  </si>
+  <si>
+    <t>k0033</t>
+  </si>
+  <si>
+    <t>k0034</t>
+  </si>
+  <si>
+    <t>k0035</t>
+  </si>
+  <si>
+    <t>k0036</t>
+  </si>
+  <si>
+    <t>k0037</t>
+  </si>
+  <si>
+    <t>k0038</t>
+  </si>
+  <si>
+    <t>k0039</t>
+  </si>
+  <si>
+    <t>k0040</t>
+  </si>
+  <si>
+    <t>k0041</t>
+  </si>
+  <si>
+    <t>k0042</t>
+  </si>
+  <si>
+    <t>k0043</t>
+  </si>
+  <si>
+    <t>k0044</t>
+  </si>
+  <si>
+    <t>k0045</t>
+  </si>
+  <si>
+    <t>k0046</t>
+  </si>
+  <si>
+    <t>k0047</t>
+  </si>
+  <si>
+    <t>k0048</t>
   </si>
 </sst>
 </file>
@@ -287,9 +359,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="0.000"/>
+    <numFmt numFmtId="164" formatCode="0.000"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -321,6 +393,12 @@
     <font>
       <sz val="11"/>
       <name val="Aptos"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="8">
@@ -413,7 +491,7 @@
     <xf numFmtId="1" fontId="5" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="5" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
@@ -721,7 +799,7 @@
   <sheetPr>
     <tabColor rgb="FF008080"/>
   </sheetPr>
-  <dimension ref="A1:AE70"/>
+  <dimension ref="A1:BC70"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.5703125" customWidth="1"/>
@@ -732,7 +810,7 @@
     <col min="8" max="31" width="11.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31" ht="24" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:55" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A1" s="1"/>
       <c r="B1" s="2" t="s">
         <v>0</v>
@@ -767,7 +845,7 @@
       <c r="AD1" s="1"/>
       <c r="AE1" s="1"/>
     </row>
-    <row r="2" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:55" x14ac:dyDescent="0.25">
       <c r="B2" s="3" t="s">
         <v>1</v>
       </c>
@@ -775,7 +853,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:55" x14ac:dyDescent="0.25">
       <c r="B3" s="5" t="s">
         <v>3</v>
       </c>
@@ -866,8 +944,80 @@
       <c r="AE3" s="5" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="4" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="AF3" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="AG3" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="AH3" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="AI3" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="AJ3" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="AK3" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="AL3" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="AM3" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="AN3" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="AO3" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="AP3" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="AQ3" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="AR3" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="AS3" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="AT3" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="AU3" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="AV3" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="AW3" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="AX3" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="AY3" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="AZ3" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="BA3" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="BB3" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="BC3" s="5" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="4" spans="1:55" x14ac:dyDescent="0.25">
       <c r="B4" s="6" t="s">
         <v>33</v>
       </c>
@@ -958,8 +1108,80 @@
       <c r="AE4" s="6" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="5" spans="1:31" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="AF4" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="AG4" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="AH4" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="AI4" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="AJ4" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="AK4" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="AL4" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="AM4" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="AN4" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="AO4" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="AP4" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="AQ4" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="AR4" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="AS4" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="AT4" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="AU4" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="AV4" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="AW4" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="AX4" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="AY4" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="AZ4" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="BA4" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="BB4" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="BC4" s="6" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="5" spans="1:55" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="7" t="s">
         <v>38</v>
       </c>
@@ -1005,7 +1227,7 @@
       <c r="AD5" s="7"/>
       <c r="AE5" s="7"/>
     </row>
-    <row r="6" spans="1:31" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:55" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="9" t="s">
         <v>45</v>
       </c>
@@ -1097,7 +1319,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="7" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:55" x14ac:dyDescent="0.25">
       <c r="B7" s="10" t="s">
         <v>48</v>
       </c>
@@ -1189,7 +1411,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="8" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:55" x14ac:dyDescent="0.25">
       <c r="B8" s="11"/>
       <c r="C8" s="12" t="s">
         <v>55</v>
@@ -1207,79 +1429,151 @@
         <v>58</v>
       </c>
       <c r="H8" s="15">
-        <v>0.6</v>
+        <v>0.5</v>
       </c>
       <c r="I8" s="15">
-        <v>0.6</v>
+        <v>0.5</v>
       </c>
       <c r="J8" s="15">
-        <v>0.6</v>
+        <v>0.5</v>
       </c>
       <c r="K8" s="15">
-        <v>0.6</v>
+        <v>0.5</v>
       </c>
       <c r="L8" s="15">
-        <v>0.6</v>
+        <v>0.5</v>
       </c>
       <c r="M8" s="15">
         <v>0.6</v>
       </c>
       <c r="N8" s="15">
+        <v>0.7</v>
+      </c>
+      <c r="O8" s="15">
+        <v>0.9</v>
+      </c>
+      <c r="P8" s="15">
+        <v>0.9</v>
+      </c>
+      <c r="Q8" s="15">
+        <v>0.9</v>
+      </c>
+      <c r="R8" s="15">
+        <v>0.8</v>
+      </c>
+      <c r="S8" s="15">
+        <v>0.5</v>
+      </c>
+      <c r="T8" s="15">
+        <v>0.3</v>
+      </c>
+      <c r="U8" s="15">
+        <v>0.3</v>
+      </c>
+      <c r="V8" s="15">
+        <v>0.3</v>
+      </c>
+      <c r="W8" s="15">
+        <v>0.5</v>
+      </c>
+      <c r="X8" s="15">
+        <v>0.7</v>
+      </c>
+      <c r="Y8" s="15">
+        <v>0.8</v>
+      </c>
+      <c r="Z8" s="15">
+        <v>0.8</v>
+      </c>
+      <c r="AA8" s="15">
+        <v>0.5</v>
+      </c>
+      <c r="AB8" s="15">
+        <v>0.4</v>
+      </c>
+      <c r="AC8" s="15">
+        <v>0.4</v>
+      </c>
+      <c r="AD8" s="15">
+        <v>0.4</v>
+      </c>
+      <c r="AE8" s="15">
+        <v>0.4</v>
+      </c>
+      <c r="AF8" s="15">
+        <v>0.5</v>
+      </c>
+      <c r="AG8" s="15">
+        <v>0.5</v>
+      </c>
+      <c r="AH8" s="15">
+        <v>0.5</v>
+      </c>
+      <c r="AI8" s="15">
+        <v>0.5</v>
+      </c>
+      <c r="AJ8" s="15">
+        <v>0.5</v>
+      </c>
+      <c r="AK8" s="15">
         <v>0.6</v>
       </c>
-      <c r="O8" s="15">
-        <v>0.6</v>
-      </c>
-      <c r="P8" s="15">
-        <v>0.6</v>
-      </c>
-      <c r="Q8" s="15">
-        <v>0.6</v>
-      </c>
-      <c r="R8" s="15">
-        <v>0.6</v>
-      </c>
-      <c r="S8" s="15">
-        <v>0.6</v>
-      </c>
-      <c r="T8" s="15">
-        <v>0.6</v>
-      </c>
-      <c r="U8" s="15">
-        <v>0.6</v>
-      </c>
-      <c r="V8" s="15">
-        <v>0.6</v>
-      </c>
-      <c r="W8" s="15">
-        <v>0.6</v>
-      </c>
-      <c r="X8" s="15">
-        <v>0.6</v>
-      </c>
-      <c r="Y8" s="15">
-        <v>0.6</v>
-      </c>
-      <c r="Z8" s="15">
-        <v>0.6</v>
-      </c>
-      <c r="AA8" s="15">
-        <v>0.6</v>
-      </c>
-      <c r="AB8" s="15">
-        <v>0.6</v>
-      </c>
-      <c r="AC8" s="15">
-        <v>0.6</v>
-      </c>
-      <c r="AD8" s="15">
-        <v>0.6</v>
-      </c>
-      <c r="AE8" s="15">
-        <v>0.6</v>
-      </c>
-    </row>
-    <row r="9" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="AL8" s="15">
+        <v>0.7</v>
+      </c>
+      <c r="AM8" s="15">
+        <v>0.9</v>
+      </c>
+      <c r="AN8" s="15">
+        <v>0.9</v>
+      </c>
+      <c r="AO8" s="15">
+        <v>0.9</v>
+      </c>
+      <c r="AP8" s="15">
+        <v>0.8</v>
+      </c>
+      <c r="AQ8" s="15">
+        <v>0.5</v>
+      </c>
+      <c r="AR8" s="15">
+        <v>0.3</v>
+      </c>
+      <c r="AS8" s="15">
+        <v>0.3</v>
+      </c>
+      <c r="AT8" s="15">
+        <v>0.3</v>
+      </c>
+      <c r="AU8" s="15">
+        <v>0.5</v>
+      </c>
+      <c r="AV8" s="15">
+        <v>0.7</v>
+      </c>
+      <c r="AW8" s="15">
+        <v>0.8</v>
+      </c>
+      <c r="AX8" s="15">
+        <v>0.8</v>
+      </c>
+      <c r="AY8" s="15">
+        <v>0.5</v>
+      </c>
+      <c r="AZ8" s="15">
+        <v>0.4</v>
+      </c>
+      <c r="BA8" s="15">
+        <v>0.4</v>
+      </c>
+      <c r="BB8" s="15">
+        <v>0.4</v>
+      </c>
+      <c r="BC8" s="15">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:55" x14ac:dyDescent="0.25">
       <c r="B9" s="11"/>
       <c r="C9" s="12"/>
       <c r="D9" s="12"/>
@@ -1311,7 +1605,7 @@
       <c r="AD9" s="14"/>
       <c r="AE9" s="14"/>
     </row>
-    <row r="10" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:55" x14ac:dyDescent="0.25">
       <c r="B10" s="11"/>
       <c r="C10" s="12"/>
       <c r="D10" s="12"/>
@@ -1343,7 +1637,7 @@
       <c r="AD10" s="14"/>
       <c r="AE10" s="14"/>
     </row>
-    <row r="11" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:55" x14ac:dyDescent="0.25">
       <c r="B11" s="11"/>
       <c r="C11" s="12"/>
       <c r="D11" s="12"/>
@@ -1375,7 +1669,7 @@
       <c r="AD11" s="14"/>
       <c r="AE11" s="14"/>
     </row>
-    <row r="12" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:55" x14ac:dyDescent="0.25">
       <c r="B12" s="11"/>
       <c r="C12" s="12"/>
       <c r="D12" s="12"/>
@@ -1407,7 +1701,7 @@
       <c r="AD12" s="14"/>
       <c r="AE12" s="14"/>
     </row>
-    <row r="13" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:55" x14ac:dyDescent="0.25">
       <c r="B13" s="11"/>
       <c r="C13" s="12"/>
       <c r="D13" s="12"/>
@@ -1439,7 +1733,7 @@
       <c r="AD13" s="14"/>
       <c r="AE13" s="14"/>
     </row>
-    <row r="14" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:55" x14ac:dyDescent="0.25">
       <c r="B14" s="11"/>
       <c r="C14" s="12"/>
       <c r="D14" s="12"/>
@@ -1471,7 +1765,7 @@
       <c r="AD14" s="14"/>
       <c r="AE14" s="14"/>
     </row>
-    <row r="15" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:55" x14ac:dyDescent="0.25">
       <c r="B15" s="11"/>
       <c r="C15" s="12"/>
       <c r="D15" s="12"/>
@@ -1503,7 +1797,7 @@
       <c r="AD15" s="14"/>
       <c r="AE15" s="14"/>
     </row>
-    <row r="16" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:55" x14ac:dyDescent="0.25">
       <c r="B16" s="11"/>
       <c r="C16" s="12"/>
       <c r="D16" s="12"/>
@@ -3264,6 +3558,7 @@
       <c r="AE70" s="14"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="6" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing r:id="rId1"/>
 </worksheet>

</xml_diff>